<commit_message>
new log for webflow web
</commit_message>
<xml_diff>
--- a/datas/mastersheet/Honda_62XS_Container_MasterSheet_r02.xlsx
+++ b/datas/mastersheet/Honda_62XS_Container_MasterSheet_r02.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\Tools\AutoHub\datas\mastersheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC487830-2BCE-47FB-B336-8AE94D55A3CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7C90661-3624-44A3-96DC-7B366CC5821E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{287B7087-B8C3-483B-8615-16E7FDDFEF13}"/>
   </bookViews>
@@ -3471,10 +3471,10 @@
     <t>37820-6WZ-M71</t>
   </si>
   <si>
-    <t>https://rb-pde-int.bosch.com:8881/app/ShowJob/16406</t>
-  </si>
-  <si>
-    <t>WF16408</t>
+    <t>WF16413</t>
+  </si>
+  <si>
+    <t>WF16414</t>
   </si>
 </sst>
 </file>
@@ -4312,24 +4312,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="31" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4348,7 +4330,25 @@
     <xf numFmtId="0" fontId="24" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12611,35 +12611,35 @@
     </row>
     <row r="2" spans="1:104">
       <c r="A2" s="39"/>
-      <c r="B2" s="110" t="s">
+      <c r="B2" s="119" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="110"/>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
-      <c r="F2" s="110"/>
-      <c r="G2" s="110"/>
-      <c r="H2" s="110"/>
+      <c r="C2" s="119"/>
+      <c r="D2" s="119"/>
+      <c r="E2" s="119"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="119"/>
+      <c r="H2" s="119"/>
     </row>
     <row r="3" spans="1:104" ht="4.5" customHeight="1">
       <c r="A3" s="39"/>
-      <c r="B3" s="110"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="110"/>
-      <c r="E3" s="110"/>
-      <c r="F3" s="110"/>
-      <c r="G3" s="110"/>
-      <c r="H3" s="110"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="119"/>
+      <c r="H3" s="119"/>
     </row>
     <row r="4" spans="1:104" ht="4.5" customHeight="1">
       <c r="A4" s="39"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="110"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
-      <c r="H4" s="110"/>
+      <c r="B4" s="119"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="119"/>
     </row>
     <row r="5" spans="1:104" s="41" customFormat="1" ht="18.75" customHeight="1">
       <c r="C5" s="67"/>
@@ -12689,75 +12689,75 @@
       <c r="CZ5" s="67"/>
     </row>
     <row r="6" spans="1:104" ht="18" customHeight="1">
-      <c r="B6" s="115" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="115"/>
-      <c r="D6" s="115"/>
-      <c r="E6" s="115"/>
-      <c r="F6" s="115"/>
-      <c r="G6" s="115"/>
-      <c r="H6" s="115"/>
-      <c r="I6" s="115"/>
-      <c r="J6" s="115"/>
-      <c r="K6" s="115"/>
-      <c r="L6" s="115"/>
-      <c r="M6" s="114" t="s">
+      <c r="B6" s="122" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="122"/>
+      <c r="D6" s="122"/>
+      <c r="E6" s="122"/>
+      <c r="F6" s="122"/>
+      <c r="G6" s="122"/>
+      <c r="H6" s="122"/>
+      <c r="I6" s="122"/>
+      <c r="J6" s="122"/>
+      <c r="K6" s="122"/>
+      <c r="L6" s="122"/>
+      <c r="M6" s="121" t="s">
         <v>307</v>
       </c>
-      <c r="N6" s="114"/>
-      <c r="O6" s="114" t="s">
+      <c r="N6" s="121"/>
+      <c r="O6" s="121" t="s">
         <v>308</v>
       </c>
-      <c r="P6" s="114"/>
+      <c r="P6" s="121"/>
       <c r="Q6" s="60" t="s">
         <v>349</v>
       </c>
       <c r="R6" s="60"/>
       <c r="S6" s="60"/>
-      <c r="T6" s="111" t="s">
+      <c r="T6" s="120" t="s">
         <v>101</v>
       </c>
-      <c r="U6" s="111"/>
-      <c r="V6" s="111"/>
-      <c r="W6" s="111"/>
-      <c r="X6" s="111"/>
-      <c r="Y6" s="111"/>
-      <c r="Z6" s="111"/>
-      <c r="AA6" s="111"/>
-      <c r="AB6" s="112" t="s">
+      <c r="U6" s="120"/>
+      <c r="V6" s="120"/>
+      <c r="W6" s="120"/>
+      <c r="X6" s="120"/>
+      <c r="Y6" s="120"/>
+      <c r="Z6" s="120"/>
+      <c r="AA6" s="120"/>
+      <c r="AB6" s="116" t="s">
         <v>125</v>
       </c>
-      <c r="AC6" s="112"/>
-      <c r="AD6" s="112"/>
-      <c r="AE6" s="112"/>
-      <c r="AF6" s="112"/>
-      <c r="AG6" s="112"/>
-      <c r="AH6" s="112"/>
-      <c r="AI6" s="112"/>
-      <c r="AJ6" s="112"/>
-      <c r="AK6" s="112"/>
-      <c r="AL6" s="113" t="s">
+      <c r="AC6" s="116"/>
+      <c r="AD6" s="116"/>
+      <c r="AE6" s="116"/>
+      <c r="AF6" s="116"/>
+      <c r="AG6" s="116"/>
+      <c r="AH6" s="116"/>
+      <c r="AI6" s="116"/>
+      <c r="AJ6" s="116"/>
+      <c r="AK6" s="116"/>
+      <c r="AL6" s="117" t="s">
         <v>126</v>
       </c>
-      <c r="AM6" s="113"/>
-      <c r="AN6" s="113"/>
-      <c r="AO6" s="113"/>
-      <c r="AP6" s="113"/>
-      <c r="AQ6" s="112" t="s">
+      <c r="AM6" s="117"/>
+      <c r="AN6" s="117"/>
+      <c r="AO6" s="117"/>
+      <c r="AP6" s="117"/>
+      <c r="AQ6" s="116" t="s">
         <v>141</v>
       </c>
-      <c r="AR6" s="112"/>
-      <c r="AS6" s="112"/>
-      <c r="AT6" s="112"/>
-      <c r="AU6" s="112"/>
-      <c r="AV6" s="113" t="s">
+      <c r="AR6" s="116"/>
+      <c r="AS6" s="116"/>
+      <c r="AT6" s="116"/>
+      <c r="AU6" s="116"/>
+      <c r="AV6" s="117" t="s">
         <v>165</v>
       </c>
-      <c r="AW6" s="113"/>
-      <c r="AX6" s="113"/>
-      <c r="AY6" s="113"/>
-      <c r="AZ6" s="113"/>
+      <c r="AW6" s="117"/>
+      <c r="AX6" s="117"/>
+      <c r="AY6" s="117"/>
+      <c r="AZ6" s="117"/>
       <c r="BA6" s="48"/>
       <c r="BB6" s="48"/>
       <c r="BC6" s="60" t="s">
@@ -12855,25 +12855,25 @@
       <c r="CK6" s="64">
         <v>14</v>
       </c>
-      <c r="CL6" s="119" t="s">
+      <c r="CL6" s="113" t="s">
         <v>193</v>
       </c>
-      <c r="CM6" s="120"/>
-      <c r="CN6" s="120"/>
-      <c r="CO6" s="120"/>
-      <c r="CP6" s="120"/>
-      <c r="CQ6" s="120"/>
-      <c r="CR6" s="121"/>
-      <c r="CS6" s="116" t="s">
+      <c r="CM6" s="114"/>
+      <c r="CN6" s="114"/>
+      <c r="CO6" s="114"/>
+      <c r="CP6" s="114"/>
+      <c r="CQ6" s="114"/>
+      <c r="CR6" s="115"/>
+      <c r="CS6" s="110" t="s">
         <v>373</v>
       </c>
-      <c r="CT6" s="117"/>
-      <c r="CU6" s="117"/>
-      <c r="CV6" s="117"/>
-      <c r="CW6" s="117"/>
-      <c r="CX6" s="117"/>
-      <c r="CY6" s="117"/>
-      <c r="CZ6" s="118"/>
+      <c r="CT6" s="111"/>
+      <c r="CU6" s="111"/>
+      <c r="CV6" s="111"/>
+      <c r="CW6" s="111"/>
+      <c r="CX6" s="111"/>
+      <c r="CY6" s="111"/>
+      <c r="CZ6" s="112"/>
     </row>
     <row r="7" spans="1:104" ht="114" collapsed="1">
       <c r="A7" s="66" t="s">
@@ -13059,38 +13059,38 @@
       <c r="BI7" s="65" t="s">
         <v>340</v>
       </c>
-      <c r="BJ7" s="122" t="s">
+      <c r="BJ7" s="118" t="s">
         <v>299</v>
       </c>
-      <c r="BK7" s="122"/>
-      <c r="BL7" s="122"/>
-      <c r="BM7" s="122"/>
-      <c r="BN7" s="122"/>
-      <c r="BO7" s="122"/>
-      <c r="BP7" s="122"/>
-      <c r="BQ7" s="122"/>
-      <c r="BR7" s="122"/>
-      <c r="BS7" s="122"/>
-      <c r="BT7" s="122"/>
-      <c r="BU7" s="122"/>
-      <c r="BV7" s="122"/>
-      <c r="BW7" s="122"/>
-      <c r="BX7" s="122" t="s">
+      <c r="BK7" s="118"/>
+      <c r="BL7" s="118"/>
+      <c r="BM7" s="118"/>
+      <c r="BN7" s="118"/>
+      <c r="BO7" s="118"/>
+      <c r="BP7" s="118"/>
+      <c r="BQ7" s="118"/>
+      <c r="BR7" s="118"/>
+      <c r="BS7" s="118"/>
+      <c r="BT7" s="118"/>
+      <c r="BU7" s="118"/>
+      <c r="BV7" s="118"/>
+      <c r="BW7" s="118"/>
+      <c r="BX7" s="118" t="s">
         <v>300</v>
       </c>
-      <c r="BY7" s="122"/>
-      <c r="BZ7" s="122"/>
-      <c r="CA7" s="122"/>
-      <c r="CB7" s="122"/>
-      <c r="CC7" s="122"/>
-      <c r="CD7" s="122"/>
-      <c r="CE7" s="122"/>
-      <c r="CF7" s="122"/>
-      <c r="CG7" s="122"/>
-      <c r="CH7" s="122"/>
-      <c r="CI7" s="122"/>
-      <c r="CJ7" s="122"/>
-      <c r="CK7" s="122"/>
+      <c r="BY7" s="118"/>
+      <c r="BZ7" s="118"/>
+      <c r="CA7" s="118"/>
+      <c r="CB7" s="118"/>
+      <c r="CC7" s="118"/>
+      <c r="CD7" s="118"/>
+      <c r="CE7" s="118"/>
+      <c r="CF7" s="118"/>
+      <c r="CG7" s="118"/>
+      <c r="CH7" s="118"/>
+      <c r="CI7" s="118"/>
+      <c r="CJ7" s="118"/>
+      <c r="CK7" s="118"/>
       <c r="CL7" s="48" t="s">
         <v>370</v>
       </c>
@@ -31510,12 +31510,6 @@
   </sheetData>
   <autoFilter ref="A10:CZ58" xr:uid="{03E47C1A-8C76-40C7-A467-A5F175EC7551}"/>
   <mergeCells count="13">
-    <mergeCell ref="CS6:CZ6"/>
-    <mergeCell ref="CL6:CR6"/>
-    <mergeCell ref="AQ6:AU6"/>
-    <mergeCell ref="AV6:AZ6"/>
-    <mergeCell ref="BJ7:BW7"/>
-    <mergeCell ref="BX7:CK7"/>
     <mergeCell ref="B2:H4"/>
     <mergeCell ref="T6:AA6"/>
     <mergeCell ref="AB6:AK6"/>
@@ -31523,6 +31517,12 @@
     <mergeCell ref="M6:N6"/>
     <mergeCell ref="B6:L6"/>
     <mergeCell ref="O6:P6"/>
+    <mergeCell ref="CS6:CZ6"/>
+    <mergeCell ref="CL6:CR6"/>
+    <mergeCell ref="AQ6:AU6"/>
+    <mergeCell ref="AV6:AZ6"/>
+    <mergeCell ref="BJ7:BW7"/>
+    <mergeCell ref="BX7:CK7"/>
   </mergeCells>
   <phoneticPr fontId="18"/>
   <conditionalFormatting sqref="T13:AZ13 BC13:CR13 BC16:CR16">

</xml_diff>

<commit_message>
Webfklow data sample and new test log
</commit_message>
<xml_diff>
--- a/datas/mastersheet/Honda_62XS_Container_MasterSheet_r02.xlsx
+++ b/datas/mastersheet/Honda_62XS_Container_MasterSheet_r02.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\Tools\AutoHub\datas\mastersheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D831F4-41F2-45E9-8906-14021EC527BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3453CA38-034A-458B-A531-E0C62F15A786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{287B7087-B8C3-483B-8615-16E7FDDFEF13}"/>
   </bookViews>
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3135" uniqueCount="667">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3135" uniqueCount="668">
   <si>
     <t>HONDA 62XS CONTAINER</t>
   </si>
@@ -3489,10 +3489,13 @@
     <t>MG1CS022_6WZXSC_V037_L8-2_FFV_Hi_0x_BL013_MP0_VIN_IMMO_ON.hex</t>
   </si>
   <si>
-    <t>WF16418</t>
-  </si>
-  <si>
-    <t>WF16419</t>
+    <t>WF16424</t>
+  </si>
+  <si>
+    <t>WF16425</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -4330,24 +4333,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="31" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4366,7 +4351,25 @@
     <xf numFmtId="0" fontId="24" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12629,35 +12632,35 @@
     </row>
     <row r="2" spans="1:104">
       <c r="A2" s="39"/>
-      <c r="B2" s="110" t="s">
+      <c r="B2" s="119" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="110"/>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
-      <c r="F2" s="110"/>
-      <c r="G2" s="110"/>
-      <c r="H2" s="110"/>
+      <c r="C2" s="119"/>
+      <c r="D2" s="119"/>
+      <c r="E2" s="119"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="119"/>
+      <c r="H2" s="119"/>
     </row>
     <row r="3" spans="1:104" ht="4.5" customHeight="1">
       <c r="A3" s="39"/>
-      <c r="B3" s="110"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="110"/>
-      <c r="E3" s="110"/>
-      <c r="F3" s="110"/>
-      <c r="G3" s="110"/>
-      <c r="H3" s="110"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="119"/>
+      <c r="H3" s="119"/>
     </row>
     <row r="4" spans="1:104" ht="4.5" customHeight="1">
       <c r="A4" s="39"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="110"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
-      <c r="H4" s="110"/>
+      <c r="B4" s="119"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="119"/>
     </row>
     <row r="5" spans="1:104" s="41" customFormat="1" ht="18.75" customHeight="1">
       <c r="C5" s="67"/>
@@ -12707,75 +12710,75 @@
       <c r="CZ5" s="67"/>
     </row>
     <row r="6" spans="1:104" ht="18" customHeight="1">
-      <c r="B6" s="115" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="115"/>
-      <c r="D6" s="115"/>
-      <c r="E6" s="115"/>
-      <c r="F6" s="115"/>
-      <c r="G6" s="115"/>
-      <c r="H6" s="115"/>
-      <c r="I6" s="115"/>
-      <c r="J6" s="115"/>
-      <c r="K6" s="115"/>
-      <c r="L6" s="115"/>
-      <c r="M6" s="114" t="s">
+      <c r="B6" s="122" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="122"/>
+      <c r="D6" s="122"/>
+      <c r="E6" s="122"/>
+      <c r="F6" s="122"/>
+      <c r="G6" s="122"/>
+      <c r="H6" s="122"/>
+      <c r="I6" s="122"/>
+      <c r="J6" s="122"/>
+      <c r="K6" s="122"/>
+      <c r="L6" s="122"/>
+      <c r="M6" s="121" t="s">
         <v>307</v>
       </c>
-      <c r="N6" s="114"/>
-      <c r="O6" s="114" t="s">
+      <c r="N6" s="121"/>
+      <c r="O6" s="121" t="s">
         <v>308</v>
       </c>
-      <c r="P6" s="114"/>
+      <c r="P6" s="121"/>
       <c r="Q6" s="60" t="s">
         <v>349</v>
       </c>
       <c r="R6" s="60"/>
       <c r="S6" s="60"/>
-      <c r="T6" s="111" t="s">
+      <c r="T6" s="120" t="s">
         <v>101</v>
       </c>
-      <c r="U6" s="111"/>
-      <c r="V6" s="111"/>
-      <c r="W6" s="111"/>
-      <c r="X6" s="111"/>
-      <c r="Y6" s="111"/>
-      <c r="Z6" s="111"/>
-      <c r="AA6" s="111"/>
-      <c r="AB6" s="112" t="s">
+      <c r="U6" s="120"/>
+      <c r="V6" s="120"/>
+      <c r="W6" s="120"/>
+      <c r="X6" s="120"/>
+      <c r="Y6" s="120"/>
+      <c r="Z6" s="120"/>
+      <c r="AA6" s="120"/>
+      <c r="AB6" s="116" t="s">
         <v>125</v>
       </c>
-      <c r="AC6" s="112"/>
-      <c r="AD6" s="112"/>
-      <c r="AE6" s="112"/>
-      <c r="AF6" s="112"/>
-      <c r="AG6" s="112"/>
-      <c r="AH6" s="112"/>
-      <c r="AI6" s="112"/>
-      <c r="AJ6" s="112"/>
-      <c r="AK6" s="112"/>
-      <c r="AL6" s="113" t="s">
+      <c r="AC6" s="116"/>
+      <c r="AD6" s="116"/>
+      <c r="AE6" s="116"/>
+      <c r="AF6" s="116"/>
+      <c r="AG6" s="116"/>
+      <c r="AH6" s="116"/>
+      <c r="AI6" s="116"/>
+      <c r="AJ6" s="116"/>
+      <c r="AK6" s="116"/>
+      <c r="AL6" s="117" t="s">
         <v>126</v>
       </c>
-      <c r="AM6" s="113"/>
-      <c r="AN6" s="113"/>
-      <c r="AO6" s="113"/>
-      <c r="AP6" s="113"/>
-      <c r="AQ6" s="112" t="s">
+      <c r="AM6" s="117"/>
+      <c r="AN6" s="117"/>
+      <c r="AO6" s="117"/>
+      <c r="AP6" s="117"/>
+      <c r="AQ6" s="116" t="s">
         <v>141</v>
       </c>
-      <c r="AR6" s="112"/>
-      <c r="AS6" s="112"/>
-      <c r="AT6" s="112"/>
-      <c r="AU6" s="112"/>
-      <c r="AV6" s="113" t="s">
+      <c r="AR6" s="116"/>
+      <c r="AS6" s="116"/>
+      <c r="AT6" s="116"/>
+      <c r="AU6" s="116"/>
+      <c r="AV6" s="117" t="s">
         <v>165</v>
       </c>
-      <c r="AW6" s="113"/>
-      <c r="AX6" s="113"/>
-      <c r="AY6" s="113"/>
-      <c r="AZ6" s="113"/>
+      <c r="AW6" s="117"/>
+      <c r="AX6" s="117"/>
+      <c r="AY6" s="117"/>
+      <c r="AZ6" s="117"/>
       <c r="BA6" s="48"/>
       <c r="BB6" s="48"/>
       <c r="BC6" s="60" t="s">
@@ -12873,25 +12876,25 @@
       <c r="CK6" s="64">
         <v>14</v>
       </c>
-      <c r="CL6" s="119" t="s">
+      <c r="CL6" s="113" t="s">
         <v>193</v>
       </c>
-      <c r="CM6" s="120"/>
-      <c r="CN6" s="120"/>
-      <c r="CO6" s="120"/>
-      <c r="CP6" s="120"/>
-      <c r="CQ6" s="120"/>
-      <c r="CR6" s="121"/>
-      <c r="CS6" s="116" t="s">
+      <c r="CM6" s="114"/>
+      <c r="CN6" s="114"/>
+      <c r="CO6" s="114"/>
+      <c r="CP6" s="114"/>
+      <c r="CQ6" s="114"/>
+      <c r="CR6" s="115"/>
+      <c r="CS6" s="110" t="s">
         <v>373</v>
       </c>
-      <c r="CT6" s="117"/>
-      <c r="CU6" s="117"/>
-      <c r="CV6" s="117"/>
-      <c r="CW6" s="117"/>
-      <c r="CX6" s="117"/>
-      <c r="CY6" s="117"/>
-      <c r="CZ6" s="118"/>
+      <c r="CT6" s="111"/>
+      <c r="CU6" s="111"/>
+      <c r="CV6" s="111"/>
+      <c r="CW6" s="111"/>
+      <c r="CX6" s="111"/>
+      <c r="CY6" s="111"/>
+      <c r="CZ6" s="112"/>
     </row>
     <row r="7" spans="1:104" ht="114" collapsed="1">
       <c r="A7" s="66" t="s">
@@ -13077,38 +13080,38 @@
       <c r="BI7" s="65" t="s">
         <v>340</v>
       </c>
-      <c r="BJ7" s="122" t="s">
+      <c r="BJ7" s="118" t="s">
         <v>299</v>
       </c>
-      <c r="BK7" s="122"/>
-      <c r="BL7" s="122"/>
-      <c r="BM7" s="122"/>
-      <c r="BN7" s="122"/>
-      <c r="BO7" s="122"/>
-      <c r="BP7" s="122"/>
-      <c r="BQ7" s="122"/>
-      <c r="BR7" s="122"/>
-      <c r="BS7" s="122"/>
-      <c r="BT7" s="122"/>
-      <c r="BU7" s="122"/>
-      <c r="BV7" s="122"/>
-      <c r="BW7" s="122"/>
-      <c r="BX7" s="122" t="s">
+      <c r="BK7" s="118"/>
+      <c r="BL7" s="118"/>
+      <c r="BM7" s="118"/>
+      <c r="BN7" s="118"/>
+      <c r="BO7" s="118"/>
+      <c r="BP7" s="118"/>
+      <c r="BQ7" s="118"/>
+      <c r="BR7" s="118"/>
+      <c r="BS7" s="118"/>
+      <c r="BT7" s="118"/>
+      <c r="BU7" s="118"/>
+      <c r="BV7" s="118"/>
+      <c r="BW7" s="118"/>
+      <c r="BX7" s="118" t="s">
         <v>300</v>
       </c>
-      <c r="BY7" s="122"/>
-      <c r="BZ7" s="122"/>
-      <c r="CA7" s="122"/>
-      <c r="CB7" s="122"/>
-      <c r="CC7" s="122"/>
-      <c r="CD7" s="122"/>
-      <c r="CE7" s="122"/>
-      <c r="CF7" s="122"/>
-      <c r="CG7" s="122"/>
-      <c r="CH7" s="122"/>
-      <c r="CI7" s="122"/>
-      <c r="CJ7" s="122"/>
-      <c r="CK7" s="122"/>
+      <c r="BY7" s="118"/>
+      <c r="BZ7" s="118"/>
+      <c r="CA7" s="118"/>
+      <c r="CB7" s="118"/>
+      <c r="CC7" s="118"/>
+      <c r="CD7" s="118"/>
+      <c r="CE7" s="118"/>
+      <c r="CF7" s="118"/>
+      <c r="CG7" s="118"/>
+      <c r="CH7" s="118"/>
+      <c r="CI7" s="118"/>
+      <c r="CJ7" s="118"/>
+      <c r="CK7" s="118"/>
       <c r="CL7" s="48" t="s">
         <v>370</v>
       </c>
@@ -29867,7 +29870,7 @@
         <v>405</v>
       </c>
       <c r="Y59" s="51" t="s">
-        <v>405</v>
+        <v>667</v>
       </c>
       <c r="Z59" s="51" t="s">
         <v>405</v>
@@ -30737,7 +30740,7 @@
         <v>405</v>
       </c>
       <c r="Y62" s="51" t="s">
-        <v>405</v>
+        <v>667</v>
       </c>
       <c r="Z62" s="51" t="s">
         <v>405</v>
@@ -31552,12 +31555,6 @@
   </sheetData>
   <autoFilter ref="A10:CZ58" xr:uid="{03E47C1A-8C76-40C7-A467-A5F175EC7551}"/>
   <mergeCells count="13">
-    <mergeCell ref="CS6:CZ6"/>
-    <mergeCell ref="CL6:CR6"/>
-    <mergeCell ref="AQ6:AU6"/>
-    <mergeCell ref="AV6:AZ6"/>
-    <mergeCell ref="BJ7:BW7"/>
-    <mergeCell ref="BX7:CK7"/>
     <mergeCell ref="B2:H4"/>
     <mergeCell ref="T6:AA6"/>
     <mergeCell ref="AB6:AK6"/>
@@ -31565,6 +31562,12 @@
     <mergeCell ref="M6:N6"/>
     <mergeCell ref="B6:L6"/>
     <mergeCell ref="O6:P6"/>
+    <mergeCell ref="CS6:CZ6"/>
+    <mergeCell ref="CL6:CR6"/>
+    <mergeCell ref="AQ6:AU6"/>
+    <mergeCell ref="AV6:AZ6"/>
+    <mergeCell ref="BJ7:BW7"/>
+    <mergeCell ref="BX7:CK7"/>
   </mergeCells>
   <phoneticPr fontId="18"/>
   <conditionalFormatting sqref="T13:AZ13 BC13:CR13 BC16:CR16">

</xml_diff>

<commit_message>
webflow log error for pick PST_Lib
</commit_message>
<xml_diff>
--- a/datas/mastersheet/Honda_62XS_Container_MasterSheet_r02.xlsx
+++ b/datas/mastersheet/Honda_62XS_Container_MasterSheet_r02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\Tools\AutoHub\datas\mastersheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F14C94C-BF1D-4DB4-B71A-82E74ECCC904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89F6166-B4C3-496C-95B3-9A80062EDB05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{287B7087-B8C3-483B-8615-16E7FDDFEF13}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11835" activeTab="1" xr2:uid="{287B7087-B8C3-483B-8615-16E7FDDFEF13}"/>
   </bookViews>
   <sheets>
     <sheet name="WorkFlow_Detail" sheetId="4" r:id="rId1"/>
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3135" uniqueCount="668">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3135" uniqueCount="669">
   <si>
     <t>HONDA 62XS CONTAINER</t>
   </si>
@@ -3480,9 +3480,6 @@
     <t>6WZX for MP0 event</t>
   </si>
   <si>
-    <t>MG1CS022_62XSC_V037</t>
-  </si>
-  <si>
     <t>MG1CS022_6WZXSC_V037_L8-2_FFV_Lo_0x_BL013_MP0_VIN_IMMO_ON.hex</t>
   </si>
   <si>
@@ -3496,6 +3493,12 @@
   </si>
   <si>
     <t>WF16438</t>
+  </si>
+  <si>
+    <t>MG1CS022_62XSC_V020_CS</t>
+  </si>
+  <si>
+    <t>V020</t>
   </si>
 </sst>
 </file>
@@ -4333,24 +4336,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="31" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4369,7 +4354,25 @@
     <xf numFmtId="0" fontId="24" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12632,35 +12635,35 @@
     </row>
     <row r="2" spans="1:104">
       <c r="A2" s="39"/>
-      <c r="B2" s="110" t="s">
+      <c r="B2" s="119" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="110"/>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
-      <c r="F2" s="110"/>
-      <c r="G2" s="110"/>
-      <c r="H2" s="110"/>
+      <c r="C2" s="119"/>
+      <c r="D2" s="119"/>
+      <c r="E2" s="119"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="119"/>
+      <c r="H2" s="119"/>
     </row>
     <row r="3" spans="1:104" ht="4.5" customHeight="1">
       <c r="A3" s="39"/>
-      <c r="B3" s="110"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="110"/>
-      <c r="E3" s="110"/>
-      <c r="F3" s="110"/>
-      <c r="G3" s="110"/>
-      <c r="H3" s="110"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="119"/>
+      <c r="H3" s="119"/>
     </row>
     <row r="4" spans="1:104" ht="4.5" customHeight="1">
       <c r="A4" s="39"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="110"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
-      <c r="H4" s="110"/>
+      <c r="B4" s="119"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="119"/>
     </row>
     <row r="5" spans="1:104" s="41" customFormat="1" ht="18.75" customHeight="1">
       <c r="C5" s="67"/>
@@ -12710,75 +12713,75 @@
       <c r="CZ5" s="67"/>
     </row>
     <row r="6" spans="1:104" ht="18" customHeight="1">
-      <c r="B6" s="115" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="115"/>
-      <c r="D6" s="115"/>
-      <c r="E6" s="115"/>
-      <c r="F6" s="115"/>
-      <c r="G6" s="115"/>
-      <c r="H6" s="115"/>
-      <c r="I6" s="115"/>
-      <c r="J6" s="115"/>
-      <c r="K6" s="115"/>
-      <c r="L6" s="115"/>
-      <c r="M6" s="114" t="s">
+      <c r="B6" s="122" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="122"/>
+      <c r="D6" s="122"/>
+      <c r="E6" s="122"/>
+      <c r="F6" s="122"/>
+      <c r="G6" s="122"/>
+      <c r="H6" s="122"/>
+      <c r="I6" s="122"/>
+      <c r="J6" s="122"/>
+      <c r="K6" s="122"/>
+      <c r="L6" s="122"/>
+      <c r="M6" s="121" t="s">
         <v>307</v>
       </c>
-      <c r="N6" s="114"/>
-      <c r="O6" s="114" t="s">
+      <c r="N6" s="121"/>
+      <c r="O6" s="121" t="s">
         <v>308</v>
       </c>
-      <c r="P6" s="114"/>
+      <c r="P6" s="121"/>
       <c r="Q6" s="60" t="s">
         <v>349</v>
       </c>
       <c r="R6" s="60"/>
       <c r="S6" s="60"/>
-      <c r="T6" s="111" t="s">
+      <c r="T6" s="120" t="s">
         <v>101</v>
       </c>
-      <c r="U6" s="111"/>
-      <c r="V6" s="111"/>
-      <c r="W6" s="111"/>
-      <c r="X6" s="111"/>
-      <c r="Y6" s="111"/>
-      <c r="Z6" s="111"/>
-      <c r="AA6" s="111"/>
-      <c r="AB6" s="112" t="s">
+      <c r="U6" s="120"/>
+      <c r="V6" s="120"/>
+      <c r="W6" s="120"/>
+      <c r="X6" s="120"/>
+      <c r="Y6" s="120"/>
+      <c r="Z6" s="120"/>
+      <c r="AA6" s="120"/>
+      <c r="AB6" s="116" t="s">
         <v>125</v>
       </c>
-      <c r="AC6" s="112"/>
-      <c r="AD6" s="112"/>
-      <c r="AE6" s="112"/>
-      <c r="AF6" s="112"/>
-      <c r="AG6" s="112"/>
-      <c r="AH6" s="112"/>
-      <c r="AI6" s="112"/>
-      <c r="AJ6" s="112"/>
-      <c r="AK6" s="112"/>
-      <c r="AL6" s="113" t="s">
+      <c r="AC6" s="116"/>
+      <c r="AD6" s="116"/>
+      <c r="AE6" s="116"/>
+      <c r="AF6" s="116"/>
+      <c r="AG6" s="116"/>
+      <c r="AH6" s="116"/>
+      <c r="AI6" s="116"/>
+      <c r="AJ6" s="116"/>
+      <c r="AK6" s="116"/>
+      <c r="AL6" s="117" t="s">
         <v>126</v>
       </c>
-      <c r="AM6" s="113"/>
-      <c r="AN6" s="113"/>
-      <c r="AO6" s="113"/>
-      <c r="AP6" s="113"/>
-      <c r="AQ6" s="112" t="s">
+      <c r="AM6" s="117"/>
+      <c r="AN6" s="117"/>
+      <c r="AO6" s="117"/>
+      <c r="AP6" s="117"/>
+      <c r="AQ6" s="116" t="s">
         <v>141</v>
       </c>
-      <c r="AR6" s="112"/>
-      <c r="AS6" s="112"/>
-      <c r="AT6" s="112"/>
-      <c r="AU6" s="112"/>
-      <c r="AV6" s="113" t="s">
+      <c r="AR6" s="116"/>
+      <c r="AS6" s="116"/>
+      <c r="AT6" s="116"/>
+      <c r="AU6" s="116"/>
+      <c r="AV6" s="117" t="s">
         <v>165</v>
       </c>
-      <c r="AW6" s="113"/>
-      <c r="AX6" s="113"/>
-      <c r="AY6" s="113"/>
-      <c r="AZ6" s="113"/>
+      <c r="AW6" s="117"/>
+      <c r="AX6" s="117"/>
+      <c r="AY6" s="117"/>
+      <c r="AZ6" s="117"/>
       <c r="BA6" s="48"/>
       <c r="BB6" s="48"/>
       <c r="BC6" s="60" t="s">
@@ -12876,25 +12879,25 @@
       <c r="CK6" s="64">
         <v>14</v>
       </c>
-      <c r="CL6" s="119" t="s">
+      <c r="CL6" s="113" t="s">
         <v>193</v>
       </c>
-      <c r="CM6" s="120"/>
-      <c r="CN6" s="120"/>
-      <c r="CO6" s="120"/>
-      <c r="CP6" s="120"/>
-      <c r="CQ6" s="120"/>
-      <c r="CR6" s="121"/>
-      <c r="CS6" s="116" t="s">
+      <c r="CM6" s="114"/>
+      <c r="CN6" s="114"/>
+      <c r="CO6" s="114"/>
+      <c r="CP6" s="114"/>
+      <c r="CQ6" s="114"/>
+      <c r="CR6" s="115"/>
+      <c r="CS6" s="110" t="s">
         <v>373</v>
       </c>
-      <c r="CT6" s="117"/>
-      <c r="CU6" s="117"/>
-      <c r="CV6" s="117"/>
-      <c r="CW6" s="117"/>
-      <c r="CX6" s="117"/>
-      <c r="CY6" s="117"/>
-      <c r="CZ6" s="118"/>
+      <c r="CT6" s="111"/>
+      <c r="CU6" s="111"/>
+      <c r="CV6" s="111"/>
+      <c r="CW6" s="111"/>
+      <c r="CX6" s="111"/>
+      <c r="CY6" s="111"/>
+      <c r="CZ6" s="112"/>
     </row>
     <row r="7" spans="1:104" ht="114" collapsed="1">
       <c r="A7" s="66" t="s">
@@ -13080,38 +13083,38 @@
       <c r="BI7" s="65" t="s">
         <v>340</v>
       </c>
-      <c r="BJ7" s="122" t="s">
+      <c r="BJ7" s="118" t="s">
         <v>299</v>
       </c>
-      <c r="BK7" s="122"/>
-      <c r="BL7" s="122"/>
-      <c r="BM7" s="122"/>
-      <c r="BN7" s="122"/>
-      <c r="BO7" s="122"/>
-      <c r="BP7" s="122"/>
-      <c r="BQ7" s="122"/>
-      <c r="BR7" s="122"/>
-      <c r="BS7" s="122"/>
-      <c r="BT7" s="122"/>
-      <c r="BU7" s="122"/>
-      <c r="BV7" s="122"/>
-      <c r="BW7" s="122"/>
-      <c r="BX7" s="122" t="s">
+      <c r="BK7" s="118"/>
+      <c r="BL7" s="118"/>
+      <c r="BM7" s="118"/>
+      <c r="BN7" s="118"/>
+      <c r="BO7" s="118"/>
+      <c r="BP7" s="118"/>
+      <c r="BQ7" s="118"/>
+      <c r="BR7" s="118"/>
+      <c r="BS7" s="118"/>
+      <c r="BT7" s="118"/>
+      <c r="BU7" s="118"/>
+      <c r="BV7" s="118"/>
+      <c r="BW7" s="118"/>
+      <c r="BX7" s="118" t="s">
         <v>300</v>
       </c>
-      <c r="BY7" s="122"/>
-      <c r="BZ7" s="122"/>
-      <c r="CA7" s="122"/>
-      <c r="CB7" s="122"/>
-      <c r="CC7" s="122"/>
-      <c r="CD7" s="122"/>
-      <c r="CE7" s="122"/>
-      <c r="CF7" s="122"/>
-      <c r="CG7" s="122"/>
-      <c r="CH7" s="122"/>
-      <c r="CI7" s="122"/>
-      <c r="CJ7" s="122"/>
-      <c r="CK7" s="122"/>
+      <c r="BY7" s="118"/>
+      <c r="BZ7" s="118"/>
+      <c r="CA7" s="118"/>
+      <c r="CB7" s="118"/>
+      <c r="CC7" s="118"/>
+      <c r="CD7" s="118"/>
+      <c r="CE7" s="118"/>
+      <c r="CF7" s="118"/>
+      <c r="CG7" s="118"/>
+      <c r="CH7" s="118"/>
+      <c r="CI7" s="118"/>
+      <c r="CJ7" s="118"/>
+      <c r="CK7" s="118"/>
       <c r="CL7" s="48" t="s">
         <v>370</v>
       </c>
@@ -29831,7 +29834,7 @@
         <v>661</v>
       </c>
       <c r="I59" s="78" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="J59" s="53" t="s">
         <v>645</v>
@@ -29870,7 +29873,7 @@
         <v>405</v>
       </c>
       <c r="Y59" s="51" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="Z59" s="51" t="s">
         <v>405</v>
@@ -29951,10 +29954,10 @@
         <v>0</v>
       </c>
       <c r="AY59" s="51" t="s">
+        <v>667</v>
+      </c>
+      <c r="AZ59" s="51" t="s">
         <v>662</v>
-      </c>
-      <c r="AZ59" s="51" t="s">
-        <v>663</v>
       </c>
       <c r="BA59" s="51"/>
       <c r="BB59" s="51"/>
@@ -29969,7 +29972,7 @@
         <v>646</v>
       </c>
       <c r="BF59" s="51" t="s">
-        <v>542</v>
+        <v>668</v>
       </c>
       <c r="BG59" s="51" t="s">
         <v>467</v>
@@ -30701,7 +30704,7 @@
         <v>661</v>
       </c>
       <c r="I62" s="78" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="J62" s="53" t="s">
         <v>653</v>
@@ -30740,7 +30743,7 @@
         <v>405</v>
       </c>
       <c r="Y62" s="51" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="Z62" s="51" t="s">
         <v>405</v>
@@ -30821,10 +30824,10 @@
         <v>0</v>
       </c>
       <c r="AY62" s="51" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="AZ62" s="51" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="BA62" s="51"/>
       <c r="BB62" s="51"/>
@@ -30839,7 +30842,7 @@
         <v>646</v>
       </c>
       <c r="BF62" s="51" t="s">
-        <v>542</v>
+        <v>668</v>
       </c>
       <c r="BG62" s="51" t="s">
         <v>467</v>
@@ -31555,12 +31558,6 @@
   </sheetData>
   <autoFilter ref="A10:CZ58" xr:uid="{03E47C1A-8C76-40C7-A467-A5F175EC7551}"/>
   <mergeCells count="13">
-    <mergeCell ref="CS6:CZ6"/>
-    <mergeCell ref="CL6:CR6"/>
-    <mergeCell ref="AQ6:AU6"/>
-    <mergeCell ref="AV6:AZ6"/>
-    <mergeCell ref="BJ7:BW7"/>
-    <mergeCell ref="BX7:CK7"/>
     <mergeCell ref="B2:H4"/>
     <mergeCell ref="T6:AA6"/>
     <mergeCell ref="AB6:AK6"/>
@@ -31568,6 +31565,12 @@
     <mergeCell ref="M6:N6"/>
     <mergeCell ref="B6:L6"/>
     <mergeCell ref="O6:P6"/>
+    <mergeCell ref="CS6:CZ6"/>
+    <mergeCell ref="CL6:CR6"/>
+    <mergeCell ref="AQ6:AU6"/>
+    <mergeCell ref="AV6:AZ6"/>
+    <mergeCell ref="BJ7:BW7"/>
+    <mergeCell ref="BX7:CK7"/>
   </mergeCells>
   <phoneticPr fontId="18"/>
   <conditionalFormatting sqref="T13:AZ13 BC13:CR13 BC16:CR16">

</xml_diff>